<commit_message>
Daily slate 2026-06-05 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-03.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-03.xlsx
@@ -471,13 +471,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E2" t="n">
+        <v>47</v>
+      </c>
+      <c r="F2" t="n">
         <v>46</v>
-      </c>
-      <c r="F2" t="n">
-        <v>45</v>
       </c>
       <c r="G2" t="n">
         <v>50.5</v>
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E3" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F3" t="n">
         <v>56</v>
       </c>
       <c r="G3" t="n">
-        <v>49.1</v>
+        <v>49.5</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E4" t="n">
         <v>19</v>
       </c>
       <c r="F4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G4" t="n">
-        <v>42.2</v>
+        <v>41.3</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="E5" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F5" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G5" t="n">
-        <v>51.2</v>
+        <v>52.2</v>
       </c>
     </row>
     <row r="6">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1061</v>
+        <v>1088</v>
       </c>
       <c r="E11" t="n">
-        <v>691</v>
+        <v>706</v>
       </c>
       <c r="F11" t="n">
-        <v>370</v>
+        <v>382</v>
       </c>
       <c r="G11" t="n">
-        <v>65.09999999999999</v>
+        <v>64.90000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -761,13 +761,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E12" t="n">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F12" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G12" t="n">
         <v>70.59999999999999</v>
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="E14" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F14" t="n">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="G14" t="n">
-        <v>27.3</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="E15" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F15" t="n">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="G15" t="n">
-        <v>19.1</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E16" t="n">
         <v>28</v>
       </c>
       <c r="F16" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G16" t="n">
-        <v>21.2</v>
+        <v>21.1</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4524</v>
+        <v>4647</v>
       </c>
       <c r="E17" t="n">
-        <v>979</v>
+        <v>1015</v>
       </c>
       <c r="F17" t="n">
-        <v>3545</v>
+        <v>3632</v>
       </c>
       <c r="G17" t="n">
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
     </row>
   </sheetData>
@@ -1525,16 +1525,16 @@
         <v>210</v>
       </c>
       <c r="D7" t="n">
-        <v>65.09999999999999</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>1061</v>
+        <v>1088</v>
       </c>
       <c r="F7" t="n">
         <v>70.59999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="H7" t="n">
         <v>54.3</v>
@@ -1543,40 +1543,40 @@
         <v>151</v>
       </c>
       <c r="J7" t="n">
-        <v>27.3</v>
+        <v>27</v>
       </c>
       <c r="K7" t="n">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="L7" t="n">
-        <v>19.1</v>
+        <v>19.2</v>
       </c>
       <c r="M7" t="n">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="N7" t="n">
-        <v>21.2</v>
+        <v>21.1</v>
       </c>
       <c r="O7" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P7" t="n">
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>4524</v>
+        <v>4647</v>
       </c>
       <c r="R7" t="n">
         <v>50.5</v>
       </c>
       <c r="S7" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="T7" t="n">
-        <v>42.2</v>
+        <v>41.3</v>
       </c>
       <c r="U7" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="V7" t="n">
         <v>51.1</v>
@@ -1591,16 +1591,16 @@
         <v>380</v>
       </c>
       <c r="Z7" t="n">
-        <v>49.1</v>
+        <v>49.5</v>
       </c>
       <c r="AA7" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AB7" t="n">
-        <v>51.2</v>
+        <v>52.2</v>
       </c>
       <c r="AC7" t="n">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="AD7" t="n">
         <v>61.9</v>

</xml_diff>